<commit_message>
#1 Design Updated and Deliverables Generated
</commit_message>
<xml_diff>
--- a/Design-Files/ACF_Out-v1.0/Deliverables/_BOM/Client_BOM_ACF_Out-v2.0.xlsx
+++ b/Design-Files/ACF_Out-v1.0/Deliverables/_BOM/Client_BOM_ACF_Out-v2.0.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\stephenlong-acfoutputpcb\Design-Files\ACF_Out-v1.0\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\aSim Data\GitHub\stephenlong-acfoutputpcb\Design-Files\ACF_Out-v1.0\Deliverables\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE89D00C-A3F4-4D5D-A94B-0658EC03151B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="119">
   <si>
     <t>#</t>
   </si>
@@ -45,7 +46,10 @@
     <t>Modular / Ethernet Connectors</t>
   </si>
   <si>
-    <t>Circular Connectors</t>
+    <t>Headers and Wire Housings</t>
+  </si>
+  <si>
+    <t>Terminal Block</t>
   </si>
   <si>
     <t>Inductor</t>
@@ -102,6 +106,9 @@
     <t>J7</t>
   </si>
   <si>
+    <t>J8</t>
+  </si>
+  <si>
     <t>L1</t>
   </si>
   <si>
@@ -162,7 +169,10 @@
     <t>Modular Connectors / Ethernet Connectors RECP CAT5e B series PCBV, 24mm FP to PCB</t>
   </si>
   <si>
-    <t>CONN RCPT FMALE 12P GOLD SOLDER</t>
+    <t>CONN HEADER R/A 8POS 3MM</t>
+  </si>
+  <si>
+    <t>TERM BLK 2POS SIDE ENTRY 5MM PCB</t>
   </si>
   <si>
     <t>FIXED IND 10UH 1A 540 MOHM SMD</t>
@@ -219,9 +229,6 @@
     <t>NE8FBV-C5-LED</t>
   </si>
   <si>
-    <t>RTS714ND12S0332</t>
-  </si>
-  <si>
     <t>IND-1008 (2520 Metric)</t>
   </si>
   <si>
@@ -264,6 +271,9 @@
     <t>SM712</t>
   </si>
   <si>
+    <t>43045-0800</t>
+  </si>
+  <si>
     <t>VLS252012HBX-100M-1</t>
   </si>
   <si>
@@ -309,7 +319,7 @@
     <t>Neutrik</t>
   </si>
   <si>
-    <t>Amphenol Sine Systems</t>
+    <t>Molex</t>
   </si>
   <si>
     <t>TDK</t>
@@ -324,6 +334,9 @@
     <t>Texas Instruments</t>
   </si>
   <si>
+    <t>Comment</t>
+  </si>
+  <si>
     <t>22uF</t>
   </si>
   <si>
@@ -345,6 +358,12 @@
     <t>10uH</t>
   </si>
   <si>
+    <t>Emerald</t>
+  </si>
+  <si>
+    <t>Yellow</t>
+  </si>
+  <si>
     <t>49.9R</t>
   </si>
   <si>
@@ -358,24 +377,12 @@
   </si>
   <si>
     <t>Quantity</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Custom</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -860,24 +867,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -888,9 +894,8 @@
       <c r="H1" s="2"/>
       <c r="I1" s="14"/>
       <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -899,31 +904,28 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -933,61 +935,59 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
       </c>
-      <c r="K3" s="7"/>
-    </row>
-    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B22" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B24" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
       </c>
-      <c r="K4" s="9"/>
-    </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -997,29 +997,28 @@
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="J5" s="7">
         <v>2</v>
       </c>
-      <c r="K5" s="7"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1029,29 +1028,28 @@
         <v>2</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="J6" s="9">
         <v>4</v>
       </c>
-      <c r="K6" s="9"/>
-    </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1061,29 +1059,28 @@
         <v>2</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="J7" s="7">
         <v>2</v>
       </c>
-      <c r="K7" s="7"/>
-    </row>
-    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -1093,29 +1090,28 @@
         <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="J8" s="9">
         <v>2</v>
       </c>
-      <c r="K8" s="9"/>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1125,29 +1121,28 @@
         <v>4</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="J9" s="7">
         <v>2</v>
       </c>
-      <c r="K9" s="7"/>
-    </row>
-    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -1157,29 +1152,28 @@
         <v>5</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>115</v>
+        <v>65</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>116</v>
+        <v>65</v>
       </c>
       <c r="J10" s="9">
         <v>2</v>
       </c>
-      <c r="K10" s="9"/>
-    </row>
-    <row r="11" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:10" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1189,29 +1183,28 @@
         <v>6</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>115</v>
+        <v>47</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>66</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="I11" s="10" t="s">
-        <v>116</v>
+        <v>98</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>66</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
       </c>
-      <c r="K11" s="7"/>
-    </row>
-    <row r="12" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
@@ -1221,29 +1214,28 @@
         <v>5</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>115</v>
+        <v>67</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>116</v>
+        <v>67</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
       </c>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1253,29 +1245,28 @@
         <v>7</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>115</v>
+        <v>48</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>68</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="I13" s="10" t="s">
-        <v>116</v>
+        <v>98</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>68</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
       </c>
-      <c r="K13" s="7"/>
-    </row>
-    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:10" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
@@ -1285,29 +1276,28 @@
         <v>8</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>115</v>
+        <v>49</v>
+      </c>
+      <c r="F14" s="9">
+        <v>430450800</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>116</v>
+        <v>83</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
       </c>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -1317,29 +1307,24 @@
         <v>9</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>107</v>
+        <v>50</v>
+      </c>
+      <c r="F15" s="7">
+        <v>691137710002</v>
+      </c>
+      <c r="G15" s="8"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="8">
+        <v>691137710002</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
       </c>
-      <c r="K15" s="7"/>
-    </row>
-    <row r="16" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
@@ -1349,61 +1334,59 @@
         <v>10</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="J16" s="9">
-        <v>2</v>
-      </c>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
         <v>15</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="I17" s="10" t="s">
-        <v>116</v>
+        <v>101</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>112</v>
       </c>
       <c r="J17" s="7">
         <v>2</v>
       </c>
-      <c r="K17" s="7"/>
-    </row>
-    <row r="18" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1413,155 +1396,152 @@
         <v>11</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="J18" s="9">
-        <v>18</v>
-      </c>
-      <c r="K18" s="9"/>
-    </row>
-    <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
         <v>17</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="J19" s="7">
-        <v>8</v>
-      </c>
-      <c r="K19" s="7"/>
-    </row>
-    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="J20" s="9">
         <v>8</v>
       </c>
-      <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
         <v>19</v>
       </c>
-      <c r="C21" s="12"/>
+      <c r="C21" s="12" t="s">
+        <v>12</v>
+      </c>
       <c r="D21" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="J21" s="7">
-        <v>4</v>
-      </c>
-      <c r="K21" s="7"/>
-    </row>
-    <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J22" s="9">
-        <v>2</v>
-      </c>
-      <c r="K22" s="9"/>
-    </row>
-    <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -1571,31 +1551,61 @@
         <v>13</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="I23" s="10" t="s">
-        <v>116</v>
+        <v>102</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>91</v>
       </c>
       <c r="J23" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="1"/>
+      <c r="B24" s="11">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="G24" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="I24" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="J24" s="9">
         <v>1</v>
       </c>
-      <c r="K23" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>